<commit_message>
Dual arduino stroboscope control
</commit_message>
<xml_diff>
--- a/Stroboscope/Calculator.xlsx
+++ b/Stroboscope/Calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\monis\Documents\Arduino\SVP Project\Stroboscope\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E89FCA25-D1F1-45F5-A002-F290393043E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9DD6B08-E185-4F1C-88C9-7A35B5B806D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{DC01E61C-4B42-41C5-8F66-5370862C4211}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>RPM</t>
   </si>
@@ -75,6 +75,24 @@
   </si>
   <si>
     <t>Total step period (rounded)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angular velocity </t>
+  </si>
+  <si>
+    <t>Velocity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distance </t>
+  </si>
+  <si>
+    <t>meters</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error </t>
   </si>
 </sst>
 </file>
@@ -460,10 +478,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{956D484C-EE30-4DA9-9F1C-AFABAB0BA5B5}">
-  <dimension ref="B4:I11"/>
+  <dimension ref="B4:I17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="15.77734375" customWidth="1"/>
     <col min="5" max="5" width="25.88671875" customWidth="1"/>
     <col min="8" max="8" width="24.109375" customWidth="1"/>
   </cols>
@@ -564,6 +583,54 @@
         <v>124</v>
       </c>
     </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H12" t="s">
+        <v>17</v>
+      </c>
+      <c r="I12">
+        <f xml:space="preserve"> 54200-49600</f>
+        <v>4600</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14">
+        <f>(C4*2*PI())/60</f>
+        <v>31.415926535897931</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15">
+        <f>C14*0.04</f>
+        <v>1.2566370614359172</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16">
+        <f>C15*0.0002</f>
+        <v>2.5132741228718348E-4</v>
+      </c>
+      <c r="D16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C17" s="1">
+        <f>C16*1000</f>
+        <v>0.25132741228718347</v>
+      </c>
+      <c r="D17" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Attempted natural frequency test using AccelStepper.h (Failed)
</commit_message>
<xml_diff>
--- a/Stroboscope/Calculator.xlsx
+++ b/Stroboscope/Calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\monis\Documents\Arduino\SVP Project\Stroboscope\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9DD6B08-E185-4F1C-88C9-7A35B5B806D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99CDEE1E-7882-4044-A608-D8291158EE5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{DC01E61C-4B42-41C5-8F66-5370862C4211}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>RPM</t>
   </si>
@@ -90,9 +90,6 @@
   </si>
   <si>
     <t>mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Error </t>
   </si>
 </sst>
 </file>
@@ -108,7 +105,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -127,6 +124,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -140,10 +143,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -546,7 +550,7 @@
       <c r="B8" t="s">
         <v>5</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="3">
         <f>ROUNDDOWN(C7/2,0)</f>
         <v>62</v>
       </c>
@@ -581,15 +585,6 @@
       <c r="C11">
         <f>C8*2</f>
         <v>124</v>
-      </c>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="H12" t="s">
-        <v>17</v>
-      </c>
-      <c r="I12">
-        <f xml:space="preserve"> 54200-49600</f>
-        <v>4600</v>
       </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.3">

</xml_diff>